<commit_message>
fix: SKU regex — allow suffix without space (DE202AA, DE120AAAA etc.)
Regex was requiring \s+ before suffix so DE202AA didn't match → pack_size=None → to_ship=0.
Changed to \s* so both "DE202 AA" and "DE202AA" work correctly.

https://claude.ai/code/session_01S6KfgkMWqVsEPx2VisNB5z
</commit_message>
<xml_diff>
--- a/docs/wb_fbo_2026-04-23.xlsx
+++ b/docs/wb_fbo_2026-04-23.xlsx
@@ -534,13 +534,9 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE202AA</t>
-        </is>
-      </c>
+        <v>432</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -602,13 +598,9 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE120AAAA</t>
-        </is>
-      </c>
+        <v>288</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -640,11 +632,7 @@
       <c r="G6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE206AA</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -712,11 +700,7 @@
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE203AA</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -746,13 +730,9 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE201AA</t>
-        </is>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -784,11 +764,7 @@
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE116AAAA</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -818,11 +794,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0</v>
+        <v>288</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE119AA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -854,11 +830,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE205AA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -1020,11 +996,7 @@
       <c r="G17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE105AAAA</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1056,11 +1028,7 @@
       <c r="G18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE107AAAA</t>
-        </is>
-      </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1328,11 +1296,7 @@
       <c r="G26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE116AA</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1364,11 +1328,7 @@
       <c r="G27" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE122AAAA</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1464,11 +1424,7 @@
       <c r="G30" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE118AAAA</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1536,11 +1492,7 @@
       <c r="G32" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE106AAAA</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1572,11 +1524,7 @@
       <c r="G33" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE123AAAA</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1640,11 +1588,7 @@
       <c r="G35" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE110AAAA</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1676,11 +1620,7 @@
       <c r="G36" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE123AA</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1709,12 +1649,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G37" s="2" t="n">
-        <v>0</v>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>36 ⚠️</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE207AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -1813,12 +1755,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G40" s="2" t="n">
-        <v>0</v>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>36 ⚠️</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE208AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -1849,12 +1793,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G41" s="2" t="n">
-        <v>0</v>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE120AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -1888,11 +1834,7 @@
       <c r="G42" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE121AAAA</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1962,7 +1904,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE105DE105</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2192,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE124DE124</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2250,7 @@
       </c>
       <c r="F54" s="6" t="inlineStr"/>
       <c r="G54" s="6" t="n">
-        <v>432</v>
+        <v>1980</v>
       </c>
       <c r="H54" s="6" t="inlineStr"/>
     </row>
@@ -2339,12 +2281,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G55" s="2" t="n">
-        <v>0</v>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>432 ⚠️</t>
+        </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE202AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -2410,11 +2354,7 @@
       <c r="G57" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE206AA</t>
-        </is>
-      </c>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2446,11 +2386,7 @@
       <c r="G58" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE120AAAA</t>
-        </is>
-      </c>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2518,11 +2454,7 @@
       <c r="G60" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE119AA</t>
-        </is>
-      </c>
+      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2554,11 +2486,7 @@
       <c r="G61" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE203AA</t>
-        </is>
-      </c>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2590,11 +2518,7 @@
       <c r="G62" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE201AA</t>
-        </is>
-      </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2626,11 +2550,7 @@
       <c r="G63" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE205AA</t>
-        </is>
-      </c>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2662,11 +2582,7 @@
       <c r="G64" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE116AAAA</t>
-        </is>
-      </c>
+      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2772,11 +2688,7 @@
       <c r="G67" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE105AAAA</t>
-        </is>
-      </c>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2918,11 +2830,7 @@
       <c r="G71" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE107AAAA</t>
-        </is>
-      </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3058,11 +2966,7 @@
       <c r="G75" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE123AAAA</t>
-        </is>
-      </c>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3195,12 +3099,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G79" s="2" t="n">
-        <v>0</v>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE116AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -3234,11 +3140,7 @@
       <c r="G80" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE122AAAA</t>
-        </is>
-      </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3399,12 +3301,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G85" s="2" t="n">
-        <v>0</v>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>36 ⚠️</t>
+        </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE207AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -3438,11 +3342,7 @@
       <c r="G86" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE106AAAA</t>
-        </is>
-      </c>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3474,11 +3374,7 @@
       <c r="G87" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE118AAAA</t>
-        </is>
-      </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3510,11 +3406,7 @@
       <c r="G88" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE123AA</t>
-        </is>
-      </c>
+      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3582,11 +3474,7 @@
       <c r="G90" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE110AAAA</t>
-        </is>
-      </c>
+      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3615,12 +3503,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G91" s="2" t="n">
-        <v>0</v>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE120AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -3689,12 +3579,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G93" s="2" t="n">
-        <v>0</v>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>36 ⚠️</t>
+        </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE208AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -3910,7 +3802,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE121AAAA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -3963,12 +3855,12 @@
       </c>
       <c r="E101" s="6" t="inlineStr">
         <is>
-          <t>7.90</t>
+          <t>7.91</t>
         </is>
       </c>
       <c r="F101" s="6" t="inlineStr"/>
       <c r="G101" s="6" t="n">
-        <v>1152</v>
+        <v>1944</v>
       </c>
       <c r="H101" s="6" t="inlineStr"/>
     </row>
@@ -4000,13 +3892,9 @@
         </is>
       </c>
       <c r="G102" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE202AA</t>
-        </is>
-      </c>
+        <v>288</v>
+      </c>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4072,11 +3960,11 @@
         </is>
       </c>
       <c r="G104" s="2" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE120AAAA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -4143,12 +4031,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G106" s="2" t="n">
-        <v>0</v>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>108 ⚠️</t>
+        </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE206AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -4179,12 +4069,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G107" s="2" t="n">
-        <v>0</v>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>72 ⚠️</t>
+        </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE203AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -4215,12 +4107,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G108" s="2" t="n">
-        <v>0</v>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE116AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -4252,11 +4146,11 @@
         </is>
       </c>
       <c r="G109" s="2" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE119AA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -4287,12 +4181,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G110" s="2" t="n">
-        <v>0</v>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>72 ⚠️</t>
+        </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE201AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -4362,11 +4258,7 @@
       <c r="G112" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE205AA</t>
-        </is>
-      </c>
+      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4434,11 +4326,7 @@
       <c r="G114" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE107AAAA</t>
-        </is>
-      </c>
+      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4467,12 +4355,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G115" s="2" t="n">
-        <v>0</v>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE105AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -4680,11 +4570,7 @@
       <c r="G121" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H121" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE116AA</t>
-        </is>
-      </c>
+      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4892,11 +4778,11 @@
         </is>
       </c>
       <c r="G127" s="2" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE122AAAA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -4927,12 +4813,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G128" s="2" t="n">
-        <v>0</v>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>36 ⚠️</t>
+        </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE208AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -4999,12 +4887,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G130" s="2" t="n">
-        <v>0</v>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE123AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -5035,12 +4925,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G131" s="2" t="n">
-        <v>0</v>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE118AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -5074,11 +4966,7 @@
       <c r="G132" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H132" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE123AA</t>
-        </is>
-      </c>
+      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -5139,12 +5027,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G134" s="2" t="n">
-        <v>0</v>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE110AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -5175,12 +5065,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G135" s="2" t="n">
-        <v>0</v>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE120AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -5211,12 +5103,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G136" s="2" t="n">
-        <v>0</v>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>36 ⚠️</t>
+        </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE207AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -5247,12 +5141,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G137" s="2" t="n">
-        <v>0</v>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE106AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -5283,12 +5179,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G138" s="2" t="n">
-        <v>0</v>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE121AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -5614,7 +5512,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE118DE118-светло-персиковый</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -5686,7 +5584,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE204DE204</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -5780,7 +5678,7 @@
       </c>
       <c r="F152" s="6" t="inlineStr"/>
       <c r="G152" s="6" t="n">
-        <v>1944</v>
+        <v>4140</v>
       </c>
       <c r="H152" s="6" t="inlineStr"/>
     </row>
@@ -5812,11 +5710,11 @@
         </is>
       </c>
       <c r="G153" s="2" t="n">
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE202AA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -5882,11 +5780,7 @@
       <c r="G155" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H155" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE206AA</t>
-        </is>
-      </c>
+      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5916,11 +5810,11 @@
         </is>
       </c>
       <c r="G156" s="2" t="n">
-        <v>0</v>
+        <v>288</v>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE120AAAA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -5990,11 +5884,7 @@
       <c r="G158" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE201AA</t>
-        </is>
-      </c>
+      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -6026,11 +5916,7 @@
       <c r="G159" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE119AA</t>
-        </is>
-      </c>
+      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -6062,11 +5948,7 @@
       <c r="G160" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE205AA</t>
-        </is>
-      </c>
+      <c r="H160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6098,11 +5980,7 @@
       <c r="G161" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE203AA</t>
-        </is>
-      </c>
+      <c r="H161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -6134,11 +6012,7 @@
       <c r="G162" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE116AAAA</t>
-        </is>
-      </c>
+      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -6342,11 +6216,7 @@
       <c r="G168" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H168" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE107AAAA</t>
-        </is>
-      </c>
+      <c r="H168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -6410,11 +6280,7 @@
       <c r="G170" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H170" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE105AAAA</t>
-        </is>
-      </c>
+      <c r="H170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -6516,11 +6382,11 @@
         </is>
       </c>
       <c r="G173" s="2" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE116AA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -6654,11 +6520,7 @@
       <c r="G177" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE122AAAA</t>
-        </is>
-      </c>
+      <c r="H177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -6690,11 +6552,7 @@
       <c r="G178" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H178" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE118AAAA</t>
-        </is>
-      </c>
+      <c r="H178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -6726,11 +6584,7 @@
       <c r="G179" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H179" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE207AA</t>
-        </is>
-      </c>
+      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -6795,12 +6649,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G181" s="2" t="n">
-        <v>0</v>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE123AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -6895,12 +6751,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G184" s="2" t="n">
-        <v>0</v>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE106AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -7002,11 +6860,7 @@
       <c r="G187" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE110AAAA</t>
-        </is>
-      </c>
+      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -7035,12 +6889,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G188" s="2" t="n">
-        <v>0</v>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE123AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -7074,11 +6930,7 @@
       <c r="G189" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE208AA</t>
-        </is>
-      </c>
+      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -7110,11 +6962,7 @@
       <c r="G190" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE121AAAA</t>
-        </is>
-      </c>
+      <c r="H190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -7146,11 +6994,7 @@
       <c r="G191" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE120AA</t>
-        </is>
-      </c>
+      <c r="H191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -7220,7 +7064,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE105AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -7256,7 +7100,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE106AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7388,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE124DE124</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -7638,7 +7482,7 @@
       </c>
       <c r="F205" s="6" t="inlineStr"/>
       <c r="G205" s="6" t="n">
-        <v>1224</v>
+        <v>2628</v>
       </c>
       <c r="H205" s="6" t="inlineStr"/>
     </row>
@@ -7670,11 +7514,11 @@
         </is>
       </c>
       <c r="G206" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE202AA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -7744,11 +7588,11 @@
         </is>
       </c>
       <c r="G208" s="2" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE206AA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -7816,11 +7660,11 @@
         </is>
       </c>
       <c r="G210" s="2" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE120AAAA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -7851,12 +7695,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G211" s="2" t="n">
-        <v>0</v>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>72 ⚠️</t>
+        </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE201AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -7887,12 +7733,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G212" s="2" t="n">
-        <v>0</v>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE119AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -7924,11 +7772,11 @@
         </is>
       </c>
       <c r="G213" s="2" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>⚠️ Возможен дефицит — проверь вручную; ⚠️ Unknown pack для SKU DE205AA</t>
+          <t>⚠️ Возможен дефицит — проверь вручную</t>
         </is>
       </c>
     </row>
@@ -7997,12 +7845,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G215" s="2" t="n">
-        <v>0</v>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE107AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8033,12 +7883,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G216" s="2" t="n">
-        <v>0</v>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>36 ⚠️</t>
+        </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE203AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8069,12 +7921,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G217" s="2" t="n">
-        <v>0</v>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE116AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8105,12 +7959,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G218" s="2" t="n">
-        <v>0</v>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE116AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8179,12 +8035,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G220" s="2" t="n">
-        <v>0</v>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE105AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8585,12 +8443,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G231" s="2" t="n">
-        <v>0</v>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE110AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8621,12 +8481,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G232" s="2" t="n">
-        <v>0</v>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE122AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8695,12 +8557,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G234" s="2" t="n">
-        <v>0</v>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>36 ⚠️</t>
+        </is>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE207AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8807,12 +8671,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G237" s="2" t="n">
-        <v>0</v>
+      <c r="G237" s="2" t="inlineStr">
+        <is>
+          <t>36 ⚠️</t>
+        </is>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE208AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8881,12 +8747,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G239" s="2" t="n">
-        <v>0</v>
+      <c r="G239" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE118AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8917,12 +8785,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G240" s="2" t="n">
-        <v>0</v>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE123AA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -8953,12 +8823,14 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G241" s="2" t="n">
-        <v>0</v>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>144 ⚠️</t>
+        </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Unknown pack для SKU DE123AAAA</t>
+          <t>🔴 Товар вышел</t>
         </is>
       </c>
     </row>
@@ -9104,7 +8976,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE124DE124</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -9126,7 +8998,7 @@
       </c>
       <c r="F246" s="6" t="inlineStr"/>
       <c r="G246" s="6" t="n">
-        <v>2088</v>
+        <v>4212</v>
       </c>
       <c r="H246" s="6" t="inlineStr"/>
     </row>
@@ -9160,11 +9032,7 @@
       <c r="G247" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H247" t="inlineStr">
-        <is>
-          <t>⚠️ Unknown pack для SKU DE107AAAA</t>
-        </is>
-      </c>
+      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -9302,7 +9170,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE105AAAA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -9374,7 +9242,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE106AAAA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9422,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE110AAAA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -9770,7 +9638,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE116AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -9806,7 +9674,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE116AAAA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -9878,7 +9746,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE118AAAA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -9950,7 +9818,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE119AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10022,7 +9890,7 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE120AAAA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10058,7 +9926,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE121AAAA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10094,7 +9962,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE122AAAA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10166,7 +10034,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE123AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10202,7 +10070,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE123AAAA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10346,7 +10214,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE201AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10418,7 +10286,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE202AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10490,7 +10358,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE203AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10598,7 +10466,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE205AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10670,7 +10538,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE206AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10742,7 +10610,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>Нет продаж за 30 дней; ⚠️ Unknown pack для SKU DE207AA</t>
+          <t>Нет продаж за 30 дней</t>
         </is>
       </c>
     </row>
@@ -10814,7 +10682,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>🔴 Товар вышел; ⚠️ Продажи=0 из-за дефицита — спрос неизвестен, нужна ручная проверка; ⚠️ Unknown pack для SKU DE208AA</t>
+          <t>🔴 Товар вышел; ⚠️ Продажи=0 из-за дефицита — спрос неизвестен, нужна ручная проверка</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: ⚠️ only when total SKU stock=0 across ALL clusters, not per-cluster
https://claude.ai/code/session_01S6KfgkMWqVsEPx2VisNB5z
</commit_message>
<xml_diff>
--- a/docs/wb_fbo_2026-04-23.xlsx
+++ b/docs/wb_fbo_2026-04-23.xlsx
@@ -951,10 +951,8 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>432 ⚠️</t>
-        </is>
+      <c r="G16" s="2" t="n">
+        <v>432</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1149,10 +1147,8 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>72 ⚠️</t>
-        </is>
+      <c r="G22" s="2" t="n">
+        <v>72</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1313,10 +1309,8 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>108 ⚠️</t>
-        </is>
+      <c r="G27" s="2" t="n">
+        <v>108</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1351,10 +1345,8 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>72 ⚠️</t>
-        </is>
+      <c r="G28" s="2" t="n">
+        <v>72</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1389,10 +1381,8 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>72 ⚠️</t>
-        </is>
+      <c r="G29" s="2" t="n">
+        <v>72</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -1911,10 +1901,8 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>144 ⚠️</t>
-        </is>
+      <c r="G45" s="2" t="n">
+        <v>144</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -1985,10 +1973,8 @@
           <t>DEFICIT</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>72 ⚠️</t>
-        </is>
+      <c r="G47" s="2" t="n">
+        <v>72</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>

</xml_diff>